<commit_message>
committo qui per NTT
</commit_message>
<xml_diff>
--- a/Voti_Fantacalcio/Voti_Fantacalcio_Stagione_2023_24_Giornata_01.xlsx
+++ b/Voti_Fantacalcio/Voti_Fantacalcio_Stagione_2023_24_Giornata_01.xlsx
@@ -670,7 +670,7 @@
     <t>Burnete</t>
   </si>
   <si>
-    <t>D'aversa</t>
+    <t>D'Aversa</t>
   </si>
   <si>
     <t>Milan</t>
@@ -733,7 +733,7 @@
     <t>Di Gregorio</t>
   </si>
   <si>
-    <t>D'ambrosio</t>
+    <t>D'Ambrosio</t>
   </si>
   <si>
     <t>Pereira P.</t>
@@ -820,7 +820,7 @@
     <t>Elmas</t>
   </si>
   <si>
-    <t xml:space="preserve">Cajuste </t>
+    <t>Cajuste</t>
   </si>
   <si>
     <t>Simeone</t>
@@ -1273,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:M381"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1416,8 +1416,6 @@
       <c r="M6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
     </row>
     <row r="7">
       <c r="A7" s="0">
@@ -2173,8 +2171,6 @@
       <c r="M25" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
     </row>
     <row r="26">
       <c r="A26" s="11">
@@ -2930,8 +2926,6 @@
       <c r="M44" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
     </row>
     <row r="45">
       <c r="A45" s="0">
@@ -3687,8 +3681,6 @@
       <c r="M63" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N63" s="8"/>
-      <c r="O63" s="8"/>
     </row>
     <row r="64">
       <c r="A64" s="11">
@@ -4444,8 +4436,6 @@
       <c r="M82" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N82" s="8"/>
-      <c r="O82" s="8"/>
     </row>
     <row r="83">
       <c r="A83" s="0">
@@ -5201,8 +5191,6 @@
       <c r="M101" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N101" s="8"/>
-      <c r="O101" s="8"/>
     </row>
     <row r="102">
       <c r="A102" s="11">
@@ -5958,8 +5946,6 @@
       <c r="M120" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N120" s="8"/>
-      <c r="O120" s="8"/>
     </row>
     <row r="121">
       <c r="A121" s="0">
@@ -6633,8 +6619,6 @@
       <c r="M137" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N137" s="8"/>
-      <c r="O137" s="8"/>
     </row>
     <row r="138">
       <c r="A138" s="11">
@@ -7390,8 +7374,6 @@
       <c r="M156" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N156" s="8"/>
-      <c r="O156" s="8"/>
     </row>
     <row r="157">
       <c r="A157" s="0">
@@ -8147,8 +8129,6 @@
       <c r="M175" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N175" s="8"/>
-      <c r="O175" s="8"/>
     </row>
     <row r="176">
       <c r="A176" s="11">
@@ -8904,8 +8884,6 @@
       <c r="M194" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N194" s="8"/>
-      <c r="O194" s="8"/>
     </row>
     <row r="195">
       <c r="A195" s="0">
@@ -9661,8 +9639,6 @@
       <c r="M213" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N213" s="8"/>
-      <c r="O213" s="8"/>
     </row>
     <row r="214">
       <c r="A214" s="11">
@@ -10418,8 +10394,6 @@
       <c r="M232" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N232" s="8"/>
-      <c r="O232" s="8"/>
     </row>
     <row r="233">
       <c r="A233" s="0">
@@ -11175,8 +11149,6 @@
       <c r="M251" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N251" s="8"/>
-      <c r="O251" s="8"/>
     </row>
     <row r="252">
       <c r="A252" s="11">
@@ -11932,8 +11904,6 @@
       <c r="M270" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N270" s="8"/>
-      <c r="O270" s="8"/>
     </row>
     <row r="271">
       <c r="A271" s="0">
@@ -12689,8 +12659,6 @@
       <c r="M289" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N289" s="8"/>
-      <c r="O289" s="8"/>
     </row>
     <row r="290">
       <c r="A290" s="11">
@@ -13405,8 +13373,6 @@
       <c r="M307" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N307" s="8"/>
-      <c r="O307" s="8"/>
     </row>
     <row r="308">
       <c r="A308" s="11">
@@ -14162,8 +14128,6 @@
       <c r="M326" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N326" s="8"/>
-      <c r="O326" s="8"/>
     </row>
     <row r="327">
       <c r="A327" s="0">
@@ -14919,8 +14883,6 @@
       <c r="M345" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N345" s="8"/>
-      <c r="O345" s="8"/>
     </row>
     <row r="346">
       <c r="A346" s="11">
@@ -15676,8 +15638,6 @@
       <c r="M364" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N364" s="8"/>
-      <c r="O364" s="8"/>
     </row>
     <row r="365">
       <c r="A365" s="0">
@@ -16409,7 +16369,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:M381"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -16552,8 +16512,6 @@
       <c r="M6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
     </row>
     <row r="7">
       <c r="A7" s="0">
@@ -17309,8 +17267,6 @@
       <c r="M25" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
     </row>
     <row r="26">
       <c r="A26" s="11">
@@ -18066,8 +18022,6 @@
       <c r="M44" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
     </row>
     <row r="45">
       <c r="A45" s="0">
@@ -18823,8 +18777,6 @@
       <c r="M63" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N63" s="8"/>
-      <c r="O63" s="8"/>
     </row>
     <row r="64">
       <c r="A64" s="11">
@@ -19580,8 +19532,6 @@
       <c r="M82" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N82" s="8"/>
-      <c r="O82" s="8"/>
     </row>
     <row r="83">
       <c r="A83" s="0">
@@ -20337,8 +20287,6 @@
       <c r="M101" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N101" s="8"/>
-      <c r="O101" s="8"/>
     </row>
     <row r="102">
       <c r="A102" s="11">
@@ -21094,8 +21042,6 @@
       <c r="M120" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N120" s="8"/>
-      <c r="O120" s="8"/>
     </row>
     <row r="121">
       <c r="A121" s="0">
@@ -21769,8 +21715,6 @@
       <c r="M137" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N137" s="8"/>
-      <c r="O137" s="8"/>
     </row>
     <row r="138">
       <c r="A138" s="11">
@@ -22526,8 +22470,6 @@
       <c r="M156" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N156" s="8"/>
-      <c r="O156" s="8"/>
     </row>
     <row r="157">
       <c r="A157" s="0">
@@ -23283,8 +23225,6 @@
       <c r="M175" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N175" s="8"/>
-      <c r="O175" s="8"/>
     </row>
     <row r="176">
       <c r="A176" s="11">
@@ -24040,8 +23980,6 @@
       <c r="M194" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N194" s="8"/>
-      <c r="O194" s="8"/>
     </row>
     <row r="195">
       <c r="A195" s="0">
@@ -24797,8 +24735,6 @@
       <c r="M213" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N213" s="8"/>
-      <c r="O213" s="8"/>
     </row>
     <row r="214">
       <c r="A214" s="11">
@@ -25554,8 +25490,6 @@
       <c r="M232" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N232" s="8"/>
-      <c r="O232" s="8"/>
     </row>
     <row r="233">
       <c r="A233" s="0">
@@ -26311,8 +26245,6 @@
       <c r="M251" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N251" s="8"/>
-      <c r="O251" s="8"/>
     </row>
     <row r="252">
       <c r="A252" s="11">
@@ -27068,8 +27000,6 @@
       <c r="M270" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N270" s="8"/>
-      <c r="O270" s="8"/>
     </row>
     <row r="271">
       <c r="A271" s="0">
@@ -27825,8 +27755,6 @@
       <c r="M289" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N289" s="8"/>
-      <c r="O289" s="8"/>
     </row>
     <row r="290">
       <c r="A290" s="11">
@@ -28541,8 +28469,6 @@
       <c r="M307" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N307" s="8"/>
-      <c r="O307" s="8"/>
     </row>
     <row r="308">
       <c r="A308" s="11">
@@ -29298,8 +29224,6 @@
       <c r="M326" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N326" s="8"/>
-      <c r="O326" s="8"/>
     </row>
     <row r="327">
       <c r="A327" s="0">
@@ -30055,8 +29979,6 @@
       <c r="M345" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N345" s="8"/>
-      <c r="O345" s="8"/>
     </row>
     <row r="346">
       <c r="A346" s="11">
@@ -30812,8 +30734,6 @@
       <c r="M364" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N364" s="8"/>
-      <c r="O364" s="8"/>
     </row>
     <row r="365">
       <c r="A365" s="0">
@@ -31545,7 +31465,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:M381"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -31688,8 +31608,6 @@
       <c r="M6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
     </row>
     <row r="7">
       <c r="A7" s="0">
@@ -32445,8 +32363,6 @@
       <c r="M25" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
     </row>
     <row r="26">
       <c r="A26" s="11">
@@ -33202,8 +33118,6 @@
       <c r="M44" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
     </row>
     <row r="45">
       <c r="A45" s="0">
@@ -33959,8 +33873,6 @@
       <c r="M63" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N63" s="8"/>
-      <c r="O63" s="8"/>
     </row>
     <row r="64">
       <c r="A64" s="11">
@@ -34716,8 +34628,6 @@
       <c r="M82" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N82" s="8"/>
-      <c r="O82" s="8"/>
     </row>
     <row r="83">
       <c r="A83" s="0">
@@ -35473,8 +35383,6 @@
       <c r="M101" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N101" s="8"/>
-      <c r="O101" s="8"/>
     </row>
     <row r="102">
       <c r="A102" s="11">
@@ -36230,8 +36138,6 @@
       <c r="M120" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N120" s="8"/>
-      <c r="O120" s="8"/>
     </row>
     <row r="121">
       <c r="A121" s="0">
@@ -36905,8 +36811,6 @@
       <c r="M137" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N137" s="8"/>
-      <c r="O137" s="8"/>
     </row>
     <row r="138">
       <c r="A138" s="11">
@@ -37662,8 +37566,6 @@
       <c r="M156" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N156" s="8"/>
-      <c r="O156" s="8"/>
     </row>
     <row r="157">
       <c r="A157" s="0">
@@ -38419,8 +38321,6 @@
       <c r="M175" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N175" s="8"/>
-      <c r="O175" s="8"/>
     </row>
     <row r="176">
       <c r="A176" s="11">
@@ -39176,8 +39076,6 @@
       <c r="M194" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N194" s="8"/>
-      <c r="O194" s="8"/>
     </row>
     <row r="195">
       <c r="A195" s="0">
@@ -39933,8 +39831,6 @@
       <c r="M213" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N213" s="8"/>
-      <c r="O213" s="8"/>
     </row>
     <row r="214">
       <c r="A214" s="11">
@@ -40690,8 +40586,6 @@
       <c r="M232" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N232" s="8"/>
-      <c r="O232" s="8"/>
     </row>
     <row r="233">
       <c r="A233" s="0">
@@ -41447,8 +41341,6 @@
       <c r="M251" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N251" s="8"/>
-      <c r="O251" s="8"/>
     </row>
     <row r="252">
       <c r="A252" s="11">
@@ -42204,8 +42096,6 @@
       <c r="M270" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N270" s="8"/>
-      <c r="O270" s="8"/>
     </row>
     <row r="271">
       <c r="A271" s="0">
@@ -42961,8 +42851,6 @@
       <c r="M289" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N289" s="8"/>
-      <c r="O289" s="8"/>
     </row>
     <row r="290">
       <c r="A290" s="11">
@@ -43677,8 +43565,6 @@
       <c r="M307" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N307" s="8"/>
-      <c r="O307" s="8"/>
     </row>
     <row r="308">
       <c r="A308" s="11">
@@ -44434,8 +44320,6 @@
       <c r="M326" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N326" s="8"/>
-      <c r="O326" s="8"/>
     </row>
     <row r="327">
       <c r="A327" s="0">
@@ -45191,8 +45075,6 @@
       <c r="M345" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N345" s="8"/>
-      <c r="O345" s="8"/>
     </row>
     <row r="346">
       <c r="A346" s="11">
@@ -45948,8 +45830,6 @@
       <c r="M364" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N364" s="8"/>
-      <c r="O364" s="8"/>
     </row>
     <row r="365">
       <c r="A365" s="0">

</xml_diff>